<commit_message>
Correctifs du 10/10/2026 : frais Etsy datés et vides par défaut, non-affiliation, mentions légales, sans compteur tiers, grand prix mesuré
</commit_message>
<xml_diff>
--- a/telechargements/prix-de-revient-createur.xlsx
+++ b/telechargements/prix-de-revient-createur.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3875D832-9DE9-43F9-9890-076864803BC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEA79BD0-C41D-4D2D-BDED-897A9C757562}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -151,10 +151,10 @@
     <t>Les taux de cotisations et de frais sont à vérifier et à saisir par vous. Les valeurs fournies sont des exemples.</t>
   </si>
   <si>
-    <t>Frais Etsy pré-remplis d'après la politique de frais d'Etsy, vérifiée le 25/09/2026 : ils peuvent changer, revérifiez-les.</t>
-  </si>
-  <si>
-    <t>TVA de 20 % sur les frais Etsy, coefficient boutique, dépôt-vente : sources secondaires, à vérifier.</t>
+    <t>Frais Etsy : cellules vides, à remplir avec votre relevé Etsy (exemples du 25/09/2026 dans la colonne Aide, non vérifiés depuis). Tant qu'elles sont vides, la colonne Etsy affiche « À renseigner ».</t>
+  </si>
+  <si>
+    <t>Coefficient boutique, dépôt-vente : sources secondaires, à vérifier.</t>
   </si>
   <si>
     <t>Taux de cotisations : consultez autoentrepreneur.urssaf.fr. Ce fichier n'est pas un conseil fiscal ou comptable.</t>
@@ -283,43 +283,43 @@
     <t>Laissez 0 si vous n'en avez pas.</t>
   </si>
   <si>
-    <t>5. Etsy (frais vérifiés le 25/09/2026 sur la politique de frais d'Etsy, hors TVA)</t>
+    <t>5. Etsy (cellules VIDES : à remplir avec les frais de votre relevé Etsy, hors TVA ; page officielle : etsy.com/fr/legal/fees)</t>
   </si>
   <si>
     <t>Frais de mise en vente (USD par vente)</t>
   </si>
   <si>
-    <t>0,20 $ par annonce, renouvelée à 0,20 $ après chaque vente (etsy.com/legal/fees).</t>
+    <t>À remplir. Exemple du 25/09/2026 (non vérifié depuis) : 0,20 $ par annonce.</t>
   </si>
   <si>
     <t>Taux de conversion : 1 USD = … EUR</t>
   </si>
   <si>
-    <t>Cours BCE du 25/09/2026 (1 € = 1,1403 $). Varie avec le dollar : à mettre à jour.</t>
+    <t>À remplir (valeur d'un dollar en euros). Exemple du 25/09/2026 (cours BCE) : 0,8770 €.</t>
   </si>
   <si>
     <t>Frais de transaction (% prix + livraison)</t>
   </si>
   <si>
-    <t>6,5 % du prix + livraison + emballage cadeau (etsy.com/legal/fees).</t>
+    <t>À remplir. Exemple du 25/09/2026 (non vérifié depuis) : 6,5 % du prix + livraison.</t>
   </si>
   <si>
     <t>Frais de traitement du paiement (%)</t>
   </si>
   <si>
-    <t>4 % du total de la commande, livraison comprise (Etsy Payments, France).</t>
+    <t>À remplir. Exemple du 25/09/2026 (non vérifié depuis) : 4 % du total de la commande, livraison comprise.</t>
   </si>
   <si>
     <t>Frais de traitement du paiement fixes (€)</t>
   </si>
   <si>
-    <t>0,30 € par commande (Etsy Payments, France).</t>
-  </si>
-  <si>
-    <t>Frais réglementaires France (%)</t>
-  </si>
-  <si>
-    <t>1,14 % du prix + livraison depuis le 22/06/2026 (aide Etsy, vérifié le 25/09/2026).</t>
+    <t>À remplir. Exemple du 25/09/2026 (non vérifié depuis) : 0,30 € par commande.</t>
+  </si>
+  <si>
+    <t>Frais réglementaires (%)</t>
+  </si>
+  <si>
+    <t>À remplir : ce pourcentage dépend du pays de la boutique. Exemple du 25/09/2026 pour la France (non vérifié depuis) : 1,14 %.</t>
   </si>
   <si>
     <t>Annonce dans une autre devise que l'euro ?</t>
@@ -331,19 +331,19 @@
     <t>Frais de conversion de devise (%)</t>
   </si>
   <si>
-    <t>2,5 % du prix + livraison, seulement si l'annonce n'est pas en euros (etsy.com/legal/fees).</t>
+    <t>À remplir seulement si l'annonce n'est pas en euros. Exemple du 25/09/2026 (non vérifié depuis) : 2,5 % du prix + livraison.</t>
   </si>
   <si>
     <t>TVA facturée par Etsy sur ses frais</t>
   </si>
   <si>
-    <t>20 % (taux de source secondaire, à vérifier) : Etsy facture la TVA sur ses frais, non récupérable en franchise.</t>
+    <t>Regardez votre relevé Etsy : s'il comporte de la TVA sur les frais, saisissez son taux ici (vide = 0).</t>
   </si>
   <si>
     <t>Total des frais Etsy en % (TVA sur frais incluse)</t>
   </si>
   <si>
-    <t>S'applique au prix TTC de l'article + livraison facturée.</t>
+    <t>S'applique au prix TTC de l'article + livraison facturée. « À renseigner » tant que les frais Etsy ci-dessus sont vides : aucun prix Etsy n'est calculé avec des frais vides.</t>
   </si>
   <si>
     <t>Total des frais Etsy fixes par vente (€, TVA incluse)</t>
@@ -367,7 +367,7 @@
     <t>Prix de gros HT = prix public TTC ÷ coefficient. 2 à 2,5 selon la boutique (source secondaire, à vérifier).</t>
   </si>
   <si>
-    <t>Sources des frais Etsy (vérifiées le 25/09/2026) : etsy.com/legal/fees, etsy.com/legal/etsy-payments, aide Etsy « Regulatory Operating Fee ». TVA de 20 % sur les frais : source secondaire.</t>
+    <t>Frais Etsy : aucune valeur n'est préremplie. Les exemples de la colonne Aide ont été relevés le 25/09/2026 sur les pages publiques d'Etsy et n'ont pas été vérifiés depuis ; la page officielle (etsy.com/fr/legal/fees) et votre relevé de paiement font foi.</t>
   </si>
   <si>
     <t>Bibliothèque de matières, emballages et consommables</t>
@@ -1861,9 +1861,7 @@
       <c r="B25" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="C25" s="19">
-        <v>0.2</v>
-      </c>
+      <c r="C25" s="19"/>
       <c r="D25" s="11" t="s">
         <v>82</v>
       </c>
@@ -1872,9 +1870,7 @@
       <c r="B26" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="C26" s="20">
-        <v>0.87696220292905369</v>
-      </c>
+      <c r="C26" s="20"/>
       <c r="D26" s="11" t="s">
         <v>84</v>
       </c>
@@ -1883,20 +1879,16 @@
       <c r="B27" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="C27" s="17">
-        <v>6.5000000000000002E-2</v>
-      </c>
+      <c r="C27" s="17"/>
       <c r="D27" s="11" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" ht="24" x14ac:dyDescent="0.25">
       <c r="B28" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="C28" s="17">
-        <v>0.04</v>
-      </c>
+      <c r="C28" s="17"/>
       <c r="D28" s="11" t="s">
         <v>88</v>
       </c>
@@ -1905,20 +1897,16 @@
       <c r="B29" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C29" s="12">
-        <v>0.3</v>
-      </c>
+      <c r="C29" s="12"/>
       <c r="D29" s="11" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" ht="24" x14ac:dyDescent="0.25">
       <c r="B30" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="C30" s="17">
-        <v>1.14E-2</v>
-      </c>
+      <c r="C30" s="17"/>
       <c r="D30" s="11" t="s">
         <v>92</v>
       </c>
@@ -1934,13 +1922,11 @@
         <v>94</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" ht="24" x14ac:dyDescent="0.25">
       <c r="B32" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="C32" s="17">
-        <v>2.5000000000000001E-2</v>
-      </c>
+      <c r="C32" s="17"/>
       <c r="D32" s="11" t="s">
         <v>96</v>
       </c>
@@ -1949,20 +1935,18 @@
       <c r="B33" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="C33" s="17">
-        <v>0.2</v>
-      </c>
+      <c r="C33" s="17"/>
       <c r="D33" s="11" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" ht="24" x14ac:dyDescent="0.25">
       <c r="B34" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="C34" s="18">
-        <f>(Paramètres!$C$27+Paramètres!$C$28+Paramètres!$C$30+IF(Paramètres!$C$31="Oui",Paramètres!$C$32,0))*(1+Paramètres!$C$33)</f>
-        <v>0.13968</v>
+      <c r="C34" s="18" t="str">
+        <f>IF(OR(COUNT(Paramètres!$C$27,Paramètres!$C$28,Paramètres!$C$30)&lt;3,AND(Paramètres!$C$31="Oui",COUNT(Paramètres!$C$32)&lt;1)),"À renseigner",(Paramètres!$C$27+Paramètres!$C$28+Paramètres!$C$30+IF(Paramètres!$C$31="Oui",Paramètres!$C$32,0))*(1+N(Paramètres!$C$33)))</f>
+        <v>À renseigner</v>
       </c>
       <c r="D34" s="11" t="s">
         <v>100</v>
@@ -1972,9 +1956,9 @@
       <c r="B35" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="C35" s="14">
-        <f>(Paramètres!$C$29+Paramètres!$C$25*Paramètres!$C$26)*(1+Paramètres!$C$33)</f>
-        <v>0.57047092870297289</v>
+      <c r="C35" s="14" t="str">
+        <f>IF(COUNT(Paramètres!$C$29,Paramètres!$C$25,Paramètres!$C$26)&lt;3,"À renseigner",(Paramètres!$C$29+Paramètres!$C$25*Paramètres!$C$26)*(1+N(Paramètres!$C$33)))</f>
+        <v>À renseigner</v>
       </c>
       <c r="D35" s="11"/>
     </row>
@@ -3979,9 +3963,9 @@
         <f>Paramètres!$C$22</f>
         <v>0</v>
       </c>
-      <c r="C44" s="18">
-        <f>Paramètres!$C$34</f>
-        <v>0.13968</v>
+      <c r="C44" s="18" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),Paramètres!$C$34,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D44" s="18">
         <f>Paramètres!$C$37</f>
@@ -4000,9 +3984,9 @@
         <f>Paramètres!$C$23</f>
         <v>0</v>
       </c>
-      <c r="C45" s="14">
-        <f>Paramètres!$C$35</f>
-        <v>0.57047092870297289</v>
+      <c r="C45" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),Paramètres!$C$35,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D45" s="14">
         <f>0</f>
@@ -4021,9 +4005,9 @@
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="C46" s="14">
-        <f>$B$8</f>
-        <v>4.5999999999999996</v>
+      <c r="C46" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),$B$8,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D46" s="14">
         <f>0</f>
@@ -4042,9 +4026,9 @@
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="C47" s="14">
-        <f>$B$7</f>
-        <v>5</v>
+      <c r="C47" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),$B$7,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D47" s="14">
         <f>0</f>
@@ -4063,9 +4047,9 @@
         <f>Paramètres!$C$20-B44</f>
         <v>0.877</v>
       </c>
-      <c r="C48" s="18">
-        <f>Paramètres!$C$20-C44</f>
-        <v>0.73731999999999998</v>
+      <c r="C48" s="18" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),Paramètres!$C$20-C44,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D48" s="18">
         <f>Paramètres!$C$20-D44</f>
@@ -4084,9 +4068,9 @@
         <f>IF(B48&gt;0,($B$38+B45+B46)/B48-B47,"Taux trop élevés")</f>
         <v>13.270619536297986</v>
       </c>
-      <c r="C49" s="16">
-        <f>IF(C48&gt;0,($B$38+C45+C46)/C48-C47,"Taux trop élevés")</f>
-        <v>17.797163052726503</v>
+      <c r="C49" s="16" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),IF(C48&gt;0,($B$38+C45+C46)/C48-C47,"Taux trop élevés"),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D49" s="16">
         <f>IF(D48&gt;0,($B$38+D45+D46)/D48-D47,"Taux trop élevés")</f>
@@ -4105,9 +4089,9 @@
         <f>IF(B48&gt;0,($B$40+B45+B46)/B48-B47,"Taux trop élevés")</f>
         <v>17.251805397187383</v>
       </c>
-      <c r="C50" s="16">
-        <f>IF(C48&gt;0,($B$40+C45+C46)/C48-C47,"Taux trop élevés")</f>
-        <v>22.532556097808694</v>
+      <c r="C50" s="16" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),IF(C48&gt;0,($B$40+C45+C46)/C48-C47,"Taux trop élevés"),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D50" s="16">
         <f>IF(D48&gt;0,($B$40+D45+D46)/D48-D47,"Taux trop élevés")</f>
@@ -4171,9 +4155,9 @@
         <f>IF(ISNUMBER(B50),B50+B47,0)</f>
         <v>17.251805397187383</v>
       </c>
-      <c r="C56" s="14">
-        <f>IF(ISNUMBER(C50),C50+C47,0)</f>
-        <v>27.532556097808694</v>
+      <c r="C56" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),IF(ISNUMBER(C50),C50+C47,0),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D56" s="14">
         <f>IF(ISNUMBER(D50),D50+D47,0)</f>
@@ -4192,9 +4176,9 @@
         <f>B56-B56/(1+Paramètres!$C$19)</f>
         <v>0</v>
       </c>
-      <c r="C57" s="14">
-        <f>C56-C56/(1+Paramètres!$C$19)</f>
-        <v>0</v>
+      <c r="C57" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),C56-C56/(1+Paramètres!$C$19),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D57" s="14">
         <f>D56-D56/(1+Paramètres!$C$19)</f>
@@ -4213,9 +4197,9 @@
         <f>Paramètres!$C$16*B56/(1+Paramètres!$C$19)</f>
         <v>2.1219720638540482</v>
       </c>
-      <c r="C58" s="14">
-        <f>Paramètres!$C$16*C56/(1+Paramètres!$C$19)</f>
-        <v>3.3865044000304692</v>
+      <c r="C58" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),Paramètres!$C$16*C56/(1+Paramètres!$C$19),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D58" s="14">
         <f>Paramètres!$C$16*D56/(1+Paramètres!$C$19)</f>
@@ -4234,9 +4218,9 @@
         <f>B44*B56+IF(B56&gt;0,B45,0)</f>
         <v>0</v>
       </c>
-      <c r="C59" s="14">
-        <f>C44*C56+IF(C56&gt;0,C45,0)</f>
-        <v>4.4162183644448909</v>
+      <c r="C59" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),C44*C56+IF(C56&gt;0,C45,0),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D59" s="14">
         <f>D44*D56+IF(D56&gt;0,D45,0)</f>
@@ -4255,9 +4239,9 @@
         <f>IF(B56&gt;0,B46,0)</f>
         <v>0</v>
       </c>
-      <c r="C60" s="14">
-        <f>IF(C56&gt;0,C46,0)</f>
-        <v>4.5999999999999996</v>
+      <c r="C60" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),IF(C56&gt;0,C46,0),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D60" s="14">
         <f>IF(D56&gt;0,D46,0)</f>
@@ -4276,9 +4260,9 @@
         <f>B56-B57-B58-B59-B60</f>
         <v>15.129833333333334</v>
       </c>
-      <c r="C61" s="16">
-        <f>C56-C57-C58-C59-C60</f>
-        <v>15.129833333333336</v>
+      <c r="C61" s="16" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),C56-C57-C58-C59-C60,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D61" s="16">
         <f>D56-D57-D58-D59-D60</f>
@@ -4297,9 +4281,9 @@
         <f>B61-$B$38</f>
         <v>3.4915000000000003</v>
       </c>
-      <c r="C62" s="14">
-        <f>C61-$B$38</f>
-        <v>3.491500000000002</v>
+      <c r="C62" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),C61-$B$38,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D62" s="14">
         <f>D61-$B$38</f>
@@ -4319,8 +4303,8 @@
         <v>OK : net = net visé</v>
       </c>
       <c r="C63" s="32" t="str">
-        <f>IF(ISNUMBER(C50),IF(ABS(C61-$B$40)&lt;0.005,"OK : net = net visé","Écart à vérifier"),"Taux trop élevés")</f>
-        <v>OK : net = net visé</v>
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),IF(ISNUMBER(C50),IF(ABS(C61-$B$40)&lt;0.005,"OK : net = net visé","Écart à vérifier"),"Taux trop élevés"),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D63" s="32" t="str">
         <f>IF(ISNUMBER(D50),IF(ABS(D61-$B$40)&lt;0.005,"OK : net = net visé","Écart à vérifier"),"Taux trop élevés")</f>
@@ -5010,9 +4994,9 @@
         <f>Paramètres!$C$22</f>
         <v>0</v>
       </c>
-      <c r="C44" s="18">
-        <f>Paramètres!$C$34</f>
-        <v>0.13968</v>
+      <c r="C44" s="18" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),Paramètres!$C$34,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D44" s="18">
         <f>Paramètres!$C$37</f>
@@ -5031,9 +5015,9 @@
         <f>Paramètres!$C$23</f>
         <v>0</v>
       </c>
-      <c r="C45" s="14">
-        <f>Paramètres!$C$35</f>
-        <v>0.57047092870297289</v>
+      <c r="C45" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),Paramètres!$C$35,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D45" s="14">
         <f>0</f>
@@ -5052,9 +5036,9 @@
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="C46" s="14">
-        <f>$B$8</f>
-        <v>0</v>
+      <c r="C46" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),$B$8,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D46" s="14">
         <f>0</f>
@@ -5073,9 +5057,9 @@
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="C47" s="14">
-        <f>$B$7</f>
-        <v>0</v>
+      <c r="C47" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),$B$7,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D47" s="14">
         <f>0</f>
@@ -5094,9 +5078,9 @@
         <f>Paramètres!$C$20-B44</f>
         <v>0.877</v>
       </c>
-      <c r="C48" s="18">
-        <f>Paramètres!$C$20-C44</f>
-        <v>0.73731999999999998</v>
+      <c r="C48" s="18" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),Paramètres!$C$20-C44,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D48" s="18">
         <f>Paramètres!$C$20-D44</f>
@@ -5115,9 +5099,9 @@
         <f>IF(B48&gt;0,($B$38+B45+B46)/B48-B47,"Taux trop élevés")</f>
         <v>12.215965863005326</v>
       </c>
-      <c r="C49" s="16">
-        <f>IF(C48&gt;0,($B$38+C45+C46)/C48-C47,"Taux trop élevés")</f>
-        <v>15.303901956489236</v>
+      <c r="C49" s="16" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),IF(C48&gt;0,($B$38+C45+C46)/C48-C47,"Taux trop élevés"),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D49" s="16">
         <f>IF(D48&gt;0,($B$38+D45+D46)/D48-D47,"Taux trop élevés")</f>
@@ -5136,9 +5120,9 @@
         <f>IF(B48&gt;0,($B$40+B45+B46)/B48-B47,"Taux trop élevés")</f>
         <v>17.10235220820746</v>
       </c>
-      <c r="C50" s="16">
-        <f>IF(C48&gt;0,($B$40+C45+C46)/C48-C47,"Taux trop élevés")</f>
-        <v>21.115979242799483</v>
+      <c r="C50" s="16" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),IF(C48&gt;0,($B$40+C45+C46)/C48-C47,"Taux trop élevés"),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D50" s="16">
         <f>IF(D48&gt;0,($B$40+D45+D46)/D48-D47,"Taux trop élevés")</f>
@@ -5202,9 +5186,9 @@
         <f>IF(ISNUMBER(B50),B50+B47,0)</f>
         <v>17.10235220820746</v>
       </c>
-      <c r="C56" s="14">
-        <f>IF(ISNUMBER(C50),C50+C47,0)</f>
-        <v>21.115979242799483</v>
+      <c r="C56" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),IF(ISNUMBER(C50),C50+C47,0),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D56" s="14">
         <f>IF(ISNUMBER(D50),D50+D47,0)</f>
@@ -5223,9 +5207,9 @@
         <f>B56-B56/(1+Paramètres!$C$19)</f>
         <v>0</v>
       </c>
-      <c r="C57" s="14">
-        <f>C56-C56/(1+Paramètres!$C$19)</f>
-        <v>0</v>
+      <c r="C57" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),C56-C56/(1+Paramètres!$C$19),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D57" s="14">
         <f>D56-D56/(1+Paramètres!$C$19)</f>
@@ -5244,9 +5228,9 @@
         <f>Paramètres!$C$16*B56/(1+Paramètres!$C$19)</f>
         <v>2.1035893216095176</v>
       </c>
-      <c r="C58" s="14">
-        <f>Paramètres!$C$16*C56/(1+Paramètres!$C$19)</f>
-        <v>2.5972654468643364</v>
+      <c r="C58" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),Paramètres!$C$16*C56/(1+Paramètres!$C$19),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D58" s="14">
         <f>Paramètres!$C$16*D56/(1+Paramètres!$C$19)</f>
@@ -5265,9 +5249,9 @@
         <f>B44*B56+IF(B56&gt;0,B45,0)</f>
         <v>0</v>
       </c>
-      <c r="C59" s="14">
-        <f>C44*C56+IF(C56&gt;0,C45,0)</f>
-        <v>3.5199509093372048</v>
+      <c r="C59" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),C44*C56+IF(C56&gt;0,C45,0),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D59" s="14">
         <f>D44*D56+IF(D56&gt;0,D45,0)</f>
@@ -5286,9 +5270,9 @@
         <f>IF(B56&gt;0,B46,0)</f>
         <v>0</v>
       </c>
-      <c r="C60" s="14">
-        <f>IF(C56&gt;0,C46,0)</f>
-        <v>0</v>
+      <c r="C60" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),IF(C56&gt;0,C46,0),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D60" s="14">
         <f>IF(D56&gt;0,D46,0)</f>
@@ -5307,9 +5291,9 @@
         <f>B56-B57-B58-B59-B60</f>
         <v>14.998762886597943</v>
       </c>
-      <c r="C61" s="16">
-        <f>C56-C57-C58-C59-C60</f>
-        <v>14.998762886597941</v>
+      <c r="C61" s="16" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),C56-C57-C58-C59-C60,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D61" s="16">
         <f>D56-D57-D58-D59-D60</f>
@@ -5328,9 +5312,9 @@
         <f>B61-$B$38</f>
         <v>4.2853608247422716</v>
       </c>
-      <c r="C62" s="14">
-        <f>C61-$B$38</f>
-        <v>4.2853608247422699</v>
+      <c r="C62" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),C61-$B$38,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D62" s="14">
         <f>D61-$B$38</f>
@@ -5350,8 +5334,8 @@
         <v>OK : net = net visé</v>
       </c>
       <c r="C63" s="32" t="str">
-        <f>IF(ISNUMBER(C50),IF(ABS(C61-$B$40)&lt;0.005,"OK : net = net visé","Écart à vérifier"),"Taux trop élevés")</f>
-        <v>OK : net = net visé</v>
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),IF(ISNUMBER(C50),IF(ABS(C61-$B$40)&lt;0.005,"OK : net = net visé","Écart à vérifier"),"Taux trop élevés"),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D63" s="32" t="str">
         <f>IF(ISNUMBER(D50),IF(ABS(D61-$B$40)&lt;0.005,"OK : net = net visé","Écart à vérifier"),"Taux trop élevés")</f>
@@ -6041,9 +6025,9 @@
         <f>Paramètres!$C$22</f>
         <v>0</v>
       </c>
-      <c r="C44" s="18">
-        <f>Paramètres!$C$34</f>
-        <v>0.13968</v>
+      <c r="C44" s="18" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),Paramètres!$C$34,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D44" s="18">
         <f>Paramètres!$C$37</f>
@@ -6062,9 +6046,9 @@
         <f>Paramètres!$C$23</f>
         <v>0</v>
       </c>
-      <c r="C45" s="14">
-        <f>Paramètres!$C$35</f>
-        <v>0.57047092870297289</v>
+      <c r="C45" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),Paramètres!$C$35,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D45" s="14">
         <f>0</f>
@@ -6083,9 +6067,9 @@
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="C46" s="14">
-        <f>$B$8</f>
-        <v>0</v>
+      <c r="C46" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),$B$8,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D46" s="14">
         <f>0</f>
@@ -6104,9 +6088,9 @@
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="C47" s="14">
-        <f>$B$7</f>
-        <v>0</v>
+      <c r="C47" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),$B$7,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D47" s="14">
         <f>0</f>
@@ -6125,9 +6109,9 @@
         <f>Paramètres!$C$20-B44</f>
         <v>0.877</v>
       </c>
-      <c r="C48" s="18">
-        <f>Paramètres!$C$20-C44</f>
-        <v>0.73731999999999998</v>
+      <c r="C48" s="18" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),Paramètres!$C$20-C44,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D48" s="18">
         <f>Paramètres!$C$20-D44</f>
@@ -6146,9 +6130,9 @@
         <f>IF(B48&gt;0,($B$38+B45+B46)/B48-B47,"Taux trop élevés")</f>
         <v>6.7791460788040041</v>
       </c>
-      <c r="C49" s="16">
-        <f>IF(C48&gt;0,($B$38+C45+C46)/C48-C47,"Taux trop élevés")</f>
-        <v>8.8371155533744972</v>
+      <c r="C49" s="16" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),IF(C48&gt;0,($B$38+C45+C46)/C48-C47,"Taux trop élevés"),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D49" s="16">
         <f>IF(D48&gt;0,($B$38+D45+D46)/D48-D47,"Taux trop élevés")</f>
@@ -6167,9 +6151,9 @@
         <f>IF(B48&gt;0,($B$40+B45+B46)/B48-B47,"Taux trop élevés")</f>
         <v>9.1518472063854048</v>
       </c>
-      <c r="C50" s="16">
-        <f>IF(C48&gt;0,($B$40+C45+C46)/C48-C47,"Taux trop élevés")</f>
-        <v>11.659307937805801</v>
+      <c r="C50" s="16" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),IF(C48&gt;0,($B$40+C45+C46)/C48-C47,"Taux trop élevés"),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D50" s="16">
         <f>IF(D48&gt;0,($B$40+D45+D46)/D48-D47,"Taux trop élevés")</f>
@@ -6233,9 +6217,9 @@
         <f>IF(ISNUMBER(B50),B50+B47,0)</f>
         <v>9.1518472063854048</v>
       </c>
-      <c r="C56" s="14">
-        <f>IF(ISNUMBER(C50),C50+C47,0)</f>
-        <v>11.659307937805801</v>
+      <c r="C56" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),IF(ISNUMBER(C50),C50+C47,0),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D56" s="14">
         <f>IF(ISNUMBER(D50),D50+D47,0)</f>
@@ -6254,9 +6238,9 @@
         <f>B56-B56/(1+Paramètres!$C$19)</f>
         <v>0</v>
       </c>
-      <c r="C57" s="14">
-        <f>C56-C56/(1+Paramètres!$C$19)</f>
-        <v>0</v>
+      <c r="C57" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),C56-C56/(1+Paramètres!$C$19),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D57" s="14">
         <f>D56-D56/(1+Paramètres!$C$19)</f>
@@ -6275,9 +6259,9 @@
         <f>Paramètres!$C$16*B56/(1+Paramètres!$C$19)</f>
         <v>1.1256772063854048</v>
       </c>
-      <c r="C58" s="14">
-        <f>Paramètres!$C$16*C56/(1+Paramètres!$C$19)</f>
-        <v>1.4340948763501136</v>
+      <c r="C58" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),Paramètres!$C$16*C56/(1+Paramètres!$C$19),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D58" s="14">
         <f>Paramètres!$C$16*D56/(1+Paramètres!$C$19)</f>
@@ -6296,9 +6280,9 @@
         <f>B44*B56+IF(B56&gt;0,B45,0)</f>
         <v>0</v>
       </c>
-      <c r="C59" s="14">
-        <f>C44*C56+IF(C56&gt;0,C45,0)</f>
-        <v>2.1990430614556873</v>
+      <c r="C59" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),C44*C56+IF(C56&gt;0,C45,0),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D59" s="14">
         <f>D44*D56+IF(D56&gt;0,D45,0)</f>
@@ -6317,9 +6301,9 @@
         <f>IF(B56&gt;0,B46,0)</f>
         <v>0</v>
       </c>
-      <c r="C60" s="14">
-        <f>IF(C56&gt;0,C46,0)</f>
-        <v>0</v>
+      <c r="C60" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),IF(C56&gt;0,C46,0),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D60" s="14">
         <f>IF(D56&gt;0,D46,0)</f>
@@ -6338,9 +6322,9 @@
         <f>B56-B57-B58-B59-B60</f>
         <v>8.0261700000000005</v>
       </c>
-      <c r="C61" s="16">
-        <f>C56-C57-C58-C59-C60</f>
-        <v>8.0261700000000005</v>
+      <c r="C61" s="16" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),C56-C57-C58-C59-C60,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D61" s="16">
         <f>D56-D57-D58-D59-D60</f>
@@ -6359,9 +6343,9 @@
         <f>B61-$B$38</f>
         <v>2.0808588888888888</v>
       </c>
-      <c r="C62" s="14">
-        <f>C61-$B$38</f>
-        <v>2.0808588888888888</v>
+      <c r="C62" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),C61-$B$38,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D62" s="14">
         <f>D61-$B$38</f>
@@ -6381,8 +6365,8 @@
         <v>OK : net = net visé</v>
       </c>
       <c r="C63" s="32" t="str">
-        <f>IF(ISNUMBER(C50),IF(ABS(C61-$B$40)&lt;0.005,"OK : net = net visé","Écart à vérifier"),"Taux trop élevés")</f>
-        <v>OK : net = net visé</v>
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),IF(ISNUMBER(C50),IF(ABS(C61-$B$40)&lt;0.005,"OK : net = net visé","Écart à vérifier"),"Taux trop élevés"),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D63" s="32" t="str">
         <f>IF(ISNUMBER(D50),IF(ABS(D61-$B$40)&lt;0.005,"OK : net = net visé","Écart à vérifier"),"Taux trop élevés")</f>
@@ -7048,9 +7032,9 @@
         <f>Paramètres!$C$22</f>
         <v>0</v>
       </c>
-      <c r="C44" s="18">
-        <f>Paramètres!$C$34</f>
-        <v>0.13968</v>
+      <c r="C44" s="18" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),Paramètres!$C$34,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D44" s="18">
         <f>Paramètres!$C$37</f>
@@ -7069,9 +7053,9 @@
         <f>Paramètres!$C$23</f>
         <v>0</v>
       </c>
-      <c r="C45" s="14">
-        <f>Paramètres!$C$35</f>
-        <v>0.57047092870297289</v>
+      <c r="C45" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),Paramètres!$C$35,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D45" s="14">
         <f>0</f>
@@ -7090,9 +7074,9 @@
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="C46" s="14">
-        <f>$B$8</f>
-        <v>0</v>
+      <c r="C46" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),$B$8,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D46" s="14">
         <f>0</f>
@@ -7111,9 +7095,9 @@
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="C47" s="14">
-        <f>$B$7</f>
-        <v>0</v>
+      <c r="C47" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),$B$7,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D47" s="14">
         <f>0</f>
@@ -7132,9 +7116,9 @@
         <f>Paramètres!$C$20-B44</f>
         <v>0.877</v>
       </c>
-      <c r="C48" s="18">
-        <f>Paramètres!$C$20-C44</f>
-        <v>0.73731999999999998</v>
+      <c r="C48" s="18" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),Paramètres!$C$20-C44,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D48" s="18">
         <f>Paramètres!$C$20-D44</f>
@@ -7153,9 +7137,9 @@
         <f>IF(B48&gt;0,($B$38+B45+B46)/B48-B47,"Taux trop élevés")</f>
         <v>1.710376282782212</v>
       </c>
-      <c r="C49" s="16">
-        <f>IF(C48&gt;0,($B$38+C45+C46)/C48-C47,"Taux trop élevés")</f>
-        <v>2.808103576063274</v>
+      <c r="C49" s="16" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),IF(C48&gt;0,($B$38+C45+C46)/C48-C47,"Taux trop élevés"),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D49" s="16">
         <f>IF(D48&gt;0,($B$38+D45+D46)/D48-D47,"Taux trop élevés")</f>
@@ -7174,9 +7158,9 @@
         <f>IF(B48&gt;0,($B$40+B45+B46)/B48-B47,"Taux trop élevés")</f>
         <v>2.2234891676168758</v>
       </c>
-      <c r="C50" s="16">
-        <f>IF(C48&gt;0,($B$40+C45+C46)/C48-C47,"Taux trop élevés")</f>
-        <v>3.4184220266681669</v>
+      <c r="C50" s="16" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),IF(C48&gt;0,($B$40+C45+C46)/C48-C47,"Taux trop élevés"),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D50" s="16">
         <f>IF(D48&gt;0,($B$40+D45+D46)/D48-D47,"Taux trop élevés")</f>
@@ -7240,9 +7224,9 @@
         <f>IF(ISNUMBER(B50),B50+B47,0)</f>
         <v>2.2234891676168758</v>
       </c>
-      <c r="C56" s="14">
-        <f>IF(ISNUMBER(C50),C50+C47,0)</f>
-        <v>3.4184220266681669</v>
+      <c r="C56" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),IF(ISNUMBER(C50),C50+C47,0),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D56" s="14">
         <f>IF(ISNUMBER(D50),D50+D47,0)</f>
@@ -7261,9 +7245,9 @@
         <f>B56-B56/(1+Paramètres!$C$19)</f>
         <v>0</v>
       </c>
-      <c r="C57" s="14">
-        <f>C56-C56/(1+Paramètres!$C$19)</f>
-        <v>0</v>
+      <c r="C57" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),C56-C56/(1+Paramètres!$C$19),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D57" s="14">
         <f>D56-D56/(1+Paramètres!$C$19)</f>
@@ -7282,9 +7266,9 @@
         <f>Paramètres!$C$16*B56/(1+Paramètres!$C$19)</f>
         <v>0.27348916761687569</v>
       </c>
-      <c r="C58" s="14">
-        <f>Paramètres!$C$16*C56/(1+Paramètres!$C$19)</f>
-        <v>0.42046590928018451</v>
+      <c r="C58" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),Paramètres!$C$16*C56/(1+Paramètres!$C$19),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D58" s="14">
         <f>Paramètres!$C$16*D56/(1+Paramètres!$C$19)</f>
@@ -7303,9 +7287,9 @@
         <f>B44*B56+IF(B56&gt;0,B45,0)</f>
         <v>0</v>
       </c>
-      <c r="C59" s="14">
-        <f>C44*C56+IF(C56&gt;0,C45,0)</f>
-        <v>1.0479561173879826</v>
+      <c r="C59" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),C44*C56+IF(C56&gt;0,C45,0),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D59" s="14">
         <f>D44*D56+IF(D56&gt;0,D45,0)</f>
@@ -7324,9 +7308,9 @@
         <f>IF(B56&gt;0,B46,0)</f>
         <v>0</v>
       </c>
-      <c r="C60" s="14">
-        <f>IF(C56&gt;0,C46,0)</f>
-        <v>0</v>
+      <c r="C60" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),IF(C56&gt;0,C46,0),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D60" s="14">
         <f>IF(D56&gt;0,D46,0)</f>
@@ -7345,9 +7329,9 @@
         <f>B56-B57-B58-B59-B60</f>
         <v>1.9500000000000002</v>
       </c>
-      <c r="C61" s="16">
-        <f>C56-C57-C58-C59-C60</f>
-        <v>1.9499999999999997</v>
+      <c r="C61" s="16" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),C56-C57-C58-C59-C60,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D61" s="16">
         <f>D56-D57-D58-D59-D60</f>
@@ -7366,9 +7350,9 @@
         <f>B61-$B$38</f>
         <v>0.45000000000000018</v>
       </c>
-      <c r="C62" s="14">
-        <f>C61-$B$38</f>
-        <v>0.44999999999999973</v>
+      <c r="C62" s="14" t="str">
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),C61-$B$38,"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D62" s="14">
         <f>D61-$B$38</f>
@@ -7388,8 +7372,8 @@
         <v>OK : net = net visé</v>
       </c>
       <c r="C63" s="32" t="str">
-        <f>IF(ISNUMBER(C50),IF(ABS(C61-$B$40)&lt;0.005,"OK : net = net visé","Écart à vérifier"),"Taux trop élevés")</f>
-        <v>OK : net = net visé</v>
+        <f>IF(AND(ISNUMBER(Paramètres!$C$34),ISNUMBER(Paramètres!$C$35)),IF(ISNUMBER(C50),IF(ABS(C61-$B$40)&lt;0.005,"OK : net = net visé","Écart à vérifier"),"Taux trop élevés"),"À renseigner")</f>
+        <v>À renseigner</v>
       </c>
       <c r="D63" s="32" t="str">
         <f>IF(ISNUMBER(D50),IF(ABS(D61-$B$40)&lt;0.005,"OK : net = net visé","Écart à vérifier"),"Taux trop élevés")</f>
@@ -7600,9 +7584,9 @@
         <f>IF(AND('Fiche 1'!$B$3="",'Fiche 1'!$E$22=0,'Fiche 1'!$E$31=0,N('Fiche 1'!$B$6)=0),"",'Fiche 1'!B50)</f>
         <v>17.251805397187383</v>
       </c>
-      <c r="G5" s="16">
+      <c r="G5" s="16" t="str">
         <f>IF(AND('Fiche 1'!$B$3="",'Fiche 1'!$E$22=0,'Fiche 1'!$E$31=0,N('Fiche 1'!$B$6)=0),"",'Fiche 1'!C50)</f>
-        <v>22.532556097808694</v>
+        <v>À renseigner</v>
       </c>
       <c r="H5" s="16">
         <f>IF(AND('Fiche 1'!$B$3="",'Fiche 1'!$E$22=0,'Fiche 1'!$E$31=0,N('Fiche 1'!$B$6)=0),"",'Fiche 1'!D50)</f>
@@ -7628,9 +7612,9 @@
         <f>IF(AND('Fiche 1'!$B$3="",'Fiche 1'!$E$22=0,'Fiche 1'!$E$31=0,N('Fiche 1'!$B$6)=0),"",'Fiche 1'!B61)</f>
         <v>15.129833333333334</v>
       </c>
-      <c r="N5" s="14">
+      <c r="N5" s="14" t="str">
         <f>IF(AND('Fiche 1'!$B$3="",'Fiche 1'!$E$22=0,'Fiche 1'!$E$31=0,N('Fiche 1'!$B$6)=0),"",'Fiche 1'!C61)</f>
-        <v>15.129833333333336</v>
+        <v>À renseigner</v>
       </c>
       <c r="O5" s="14">
         <f>IF(AND('Fiche 1'!$B$3="",'Fiche 1'!$E$22=0,'Fiche 1'!$E$31=0,N('Fiche 1'!$B$6)=0),"",'Fiche 1'!D61)</f>
@@ -7677,9 +7661,9 @@
         <f>IF(AND('Fiche 2'!$B$3="",'Fiche 2'!$E$22=0,'Fiche 2'!$E$31=0,N('Fiche 2'!$B$6)=0),"",'Fiche 2'!B50)</f>
         <v>17.10235220820746</v>
       </c>
-      <c r="G6" s="16">
+      <c r="G6" s="16" t="str">
         <f>IF(AND('Fiche 2'!$B$3="",'Fiche 2'!$E$22=0,'Fiche 2'!$E$31=0,N('Fiche 2'!$B$6)=0),"",'Fiche 2'!C50)</f>
-        <v>21.115979242799483</v>
+        <v>À renseigner</v>
       </c>
       <c r="H6" s="16">
         <f>IF(AND('Fiche 2'!$B$3="",'Fiche 2'!$E$22=0,'Fiche 2'!$E$31=0,N('Fiche 2'!$B$6)=0),"",'Fiche 2'!D50)</f>
@@ -7705,9 +7689,9 @@
         <f>IF(AND('Fiche 2'!$B$3="",'Fiche 2'!$E$22=0,'Fiche 2'!$E$31=0,N('Fiche 2'!$B$6)=0),"",'Fiche 2'!B61)</f>
         <v>14.998762886597943</v>
       </c>
-      <c r="N6" s="14">
+      <c r="N6" s="14" t="str">
         <f>IF(AND('Fiche 2'!$B$3="",'Fiche 2'!$E$22=0,'Fiche 2'!$E$31=0,N('Fiche 2'!$B$6)=0),"",'Fiche 2'!C61)</f>
-        <v>14.998762886597941</v>
+        <v>À renseigner</v>
       </c>
       <c r="O6" s="14">
         <f>IF(AND('Fiche 2'!$B$3="",'Fiche 2'!$E$22=0,'Fiche 2'!$E$31=0,N('Fiche 2'!$B$6)=0),"",'Fiche 2'!D61)</f>
@@ -7754,9 +7738,9 @@
         <f>IF(AND('Fiche 3'!$B$3="",'Fiche 3'!$E$22=0,'Fiche 3'!$E$31=0,N('Fiche 3'!$B$6)=0),"",'Fiche 3'!B50)</f>
         <v>9.1518472063854048</v>
       </c>
-      <c r="G7" s="16">
+      <c r="G7" s="16" t="str">
         <f>IF(AND('Fiche 3'!$B$3="",'Fiche 3'!$E$22=0,'Fiche 3'!$E$31=0,N('Fiche 3'!$B$6)=0),"",'Fiche 3'!C50)</f>
-        <v>11.659307937805801</v>
+        <v>À renseigner</v>
       </c>
       <c r="H7" s="16">
         <f>IF(AND('Fiche 3'!$B$3="",'Fiche 3'!$E$22=0,'Fiche 3'!$E$31=0,N('Fiche 3'!$B$6)=0),"",'Fiche 3'!D50)</f>
@@ -7782,9 +7766,9 @@
         <f>IF(AND('Fiche 3'!$B$3="",'Fiche 3'!$E$22=0,'Fiche 3'!$E$31=0,N('Fiche 3'!$B$6)=0),"",'Fiche 3'!B61)</f>
         <v>8.0261700000000005</v>
       </c>
-      <c r="N7" s="14">
+      <c r="N7" s="14" t="str">
         <f>IF(AND('Fiche 3'!$B$3="",'Fiche 3'!$E$22=0,'Fiche 3'!$E$31=0,N('Fiche 3'!$B$6)=0),"",'Fiche 3'!C61)</f>
-        <v>8.0261700000000005</v>
+        <v>À renseigner</v>
       </c>
       <c r="O7" s="14">
         <f>IF(AND('Fiche 3'!$B$3="",'Fiche 3'!$E$22=0,'Fiche 3'!$E$31=0,N('Fiche 3'!$B$6)=0),"",'Fiche 3'!D61)</f>

</xml_diff>